<commit_message>
Added message for #781
</commit_message>
<xml_diff>
--- a/jeaf-generator-messages/src/main/resources/JEAFGeneratorMessages.xlsx
+++ b/jeaf-generator-messages/src/main/resources/JEAFGeneratorMessages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tillmann.schall/Projects/JEAF/jeaf-generator-messages/jeaf-generator-messages/src/main/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDFCF081-8A51-8044-B76C-7D6F7BAE686F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB4A650F-FEE4-C746-8478-7C5604C44E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25620" yWindow="640" windowWidth="51160" windowHeight="28140" activeTab="2" xr2:uid="{ADB42BFB-6EC0-410A-8CB1-9C298A092AA4}"/>
+    <workbookView xWindow="1240" yWindow="680" windowWidth="33320" windowHeight="21660" activeTab="2" xr2:uid="{ADB42BFB-6EC0-410A-8CB1-9C298A092AA4}"/>
   </bookViews>
   <sheets>
     <sheet name="Class-Info" sheetId="1" r:id="rId1"/>
@@ -281,7 +281,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="339">
   <si>
     <t>Class-Info</t>
   </si>
@@ -1300,6 +1300,15 @@
   </si>
   <si>
     <t>«CompatibilityGroup» ''{0}'' has multiple «CompatibilityInfo» definitions associated ({1}). Please make sure that there is not more than one.</t>
+  </si>
+  <si>
+    <t>TOO_MANY_INCOMPATIBLE_VERSIONS</t>
+  </si>
+  <si>
+    <t>It is possible to define the first incompatible version for a version. However, as the name implies, there is only one first incompatible first version.</t>
+  </si>
+  <si>
+    <t>«CompatibilityInfo» ''{0}'' has multiple «FirstIncomatibleVersion» dependencies. Please make sure that there is not more than one.</t>
   </si>
 </sst>
 </file>
@@ -4609,9 +4618,24 @@
         <v>335</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A90" s="1">
         <v>9188</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>338</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.2">
@@ -4670,7 +4694,7 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A101" xr:uid="{AACEF8C0-EC92-4686-A8C3-E4036D94D483}">
       <formula1>0</formula1>
     </dataValidation>
@@ -4683,7 +4707,7 @@
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="3">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EA474BAA-D9F0-48C4-BFC6-D7532DADFCD0}">
           <x14:formula1>
             <xm:f>'Predefined-Values'!$C$4:$C$5</xm:f>

</xml_diff>

<commit_message>
Added messages for #779
</commit_message>
<xml_diff>
--- a/jeaf-generator-messages/src/main/resources/JEAFGeneratorMessages.xlsx
+++ b/jeaf-generator-messages/src/main/resources/JEAFGeneratorMessages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tillmann.schall/Projects/JEAF/jeaf-generator-messages/jeaf-generator-messages/src/main/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB4A650F-FEE4-C746-8478-7C5604C44E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D5C7F22-9FAB-A64C-82F7-A7C41439234A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1240" yWindow="680" windowWidth="33320" windowHeight="21660" activeTab="2" xr2:uid="{ADB42BFB-6EC0-410A-8CB1-9C298A092AA4}"/>
+    <workbookView xWindow="69080" yWindow="3880" windowWidth="33320" windowHeight="21660" activeTab="2" xr2:uid="{ADB42BFB-6EC0-410A-8CB1-9C298A092AA4}"/>
   </bookViews>
   <sheets>
     <sheet name="Class-Info" sheetId="1" r:id="rId1"/>
@@ -281,7 +281,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="344">
   <si>
     <t>Class-Info</t>
   </si>
@@ -1309,6 +1309,21 @@
   </si>
   <si>
     <t>«CompatibilityInfo» ''{0}'' has multiple «FirstIncomatibleVersion» dependencies. Please make sure that there is not more than one.</t>
+  </si>
+  <si>
+    <t>ENUM_SUBSET_INVALID</t>
+  </si>
+  <si>
+    <t>«EnumSubset» ''{0}'' in ''{1}'' has set tags "allowedLiterals" and "notAllowedLiterals" even though only one of the must be used but not both. Please fix the UML model accordingly.</t>
+  </si>
+  <si>
+    <t>Using stereotype «EnumSubset» it is possible to limit the allowed literals for a property. This can be achieved by either using a positive or an exclusion list but not both or none.</t>
+  </si>
+  <si>
+    <t>ENUM_SUBSET_NOT_DEFINED</t>
+  </si>
+  <si>
+    <t>«EnumSubset» ''{0}'' in ''{1}'' has set not tags at all. Either "allowedLiterals" or "notAllowedLiterals" has to be but not both. Please fix the UML model accordingly.</t>
   </si>
 </sst>
 </file>
@@ -4638,14 +4653,44 @@
         <v>338</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A91" s="1">
         <v>9189</v>
       </c>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B91" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="A92" s="1">
         <v>9190</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="G92" s="1" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added error messages for #775
</commit_message>
<xml_diff>
--- a/jeaf-generator-messages/src/main/resources/JEAFGeneratorMessages.xlsx
+++ b/jeaf-generator-messages/src/main/resources/JEAFGeneratorMessages.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tillmann.schall/Projects/JEAF/jeaf-generator-messages/jeaf-generator-messages/src/main/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D5C7F22-9FAB-A64C-82F7-A7C41439234A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3A6AF03-4AE2-4741-BD9A-79294CCD56FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="69080" yWindow="3880" windowWidth="33320" windowHeight="21660" activeTab="2" xr2:uid="{ADB42BFB-6EC0-410A-8CB1-9C298A092AA4}"/>
+    <workbookView xWindow="15520" yWindow="2760" windowWidth="33320" windowHeight="21660" activeTab="2" xr2:uid="{ADB42BFB-6EC0-410A-8CB1-9C298A092AA4}"/>
   </bookViews>
   <sheets>
     <sheet name="Class-Info" sheetId="1" r:id="rId1"/>
@@ -281,7 +281,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="350">
   <si>
     <t>Class-Info</t>
   </si>
@@ -1324,6 +1324,24 @@
   </si>
   <si>
     <t>«EnumSubset» ''{0}'' in ''{1}'' has set not tags at all. Either "allowedLiterals" or "notAllowedLiterals" has to be but not both. Please fix the UML model accordingly.</t>
+  </si>
+  <si>
+    <t>MORE_THAN_ONE_COMPATIBILIY_GROUP</t>
+  </si>
+  <si>
+    <t>Model elements can be associated with «CompatibilityGroup» elements. However, at least at the moment more than one compatibioity group is not supported.</t>
+  </si>
+  <si>
+    <t>Model element ''{0}'' of ''{1}'' is associated with more that one compatibility group. Please make sure that there is not more than one depenency from the element to a «CompatibilityGroup» element in the UML model. \nReferenced Compatibility Groups: {2}</t>
+  </si>
+  <si>
+    <t>COMPATIBILITY_GROUP_HAS_NO_INFO</t>
+  </si>
+  <si>
+    <t>«CompatibilityGroup» elements always must have exactly one «CompatibilityInfo».</t>
+  </si>
+  <si>
+    <t>«CompatibilityGroup» ''{0}}'' does not have excatly one «CompatibilityInfo» element. Please fix the UML model.</t>
   </si>
 </sst>
 </file>
@@ -4693,14 +4711,44 @@
         <v>343</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="A93" s="1">
         <v>9191</v>
       </c>
-    </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B93" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A94" s="1">
         <v>9192</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F94" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="G94" s="1" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>